<commit_message>
fix: fix context application id name
</commit_message>
<xml_diff>
--- a/data/context_application_dataset_proverbs_001_100.xlsx
+++ b/data/context_application_dataset_proverbs_001_100.xlsx
@@ -40,7 +40,7 @@
     <t>correct_answer</t>
   </si>
   <si>
-    <t>P001</t>
+    <t>CAP001</t>
   </si>
   <si>
     <t>疑人，毋成賊。</t>
@@ -62,7 +62,7 @@
     <t>C</t>
   </si>
   <si>
-    <t>P002</t>
+    <t>CAP002</t>
   </si>
   <si>
     <t xml:space="preserve">校長兼摃鐘。
@@ -85,7 +85,7 @@
     <t>A</t>
   </si>
   <si>
-    <t>P003</t>
+    <t>CAP003</t>
   </si>
   <si>
     <t>無米兼閏月。</t>
@@ -109,7 +109,7 @@
     <t>時到時擔當，無米才煮番薯湯。</t>
   </si>
   <si>
-    <t>P004</t>
+    <t>CAP004</t>
   </si>
   <si>
     <t>大牛無惜力。</t>
@@ -132,7 +132,7 @@
     <t>D</t>
   </si>
   <si>
-    <t>P005</t>
+    <t>CAP005</t>
   </si>
   <si>
     <t>一時風，駛一時船。</t>
@@ -155,7 +155,7 @@
     <t>B</t>
   </si>
   <si>
-    <t>P006</t>
+    <t>CAP006</t>
   </si>
   <si>
     <t>呵咾甲會觸舌。</t>
@@ -175,7 +175,7 @@
     <t>人未到，聲先到。</t>
   </si>
   <si>
-    <t>P007</t>
+    <t>CAP007</t>
   </si>
   <si>
     <t>你看我殕殕，我看你霧霧。</t>
@@ -195,7 +195,7 @@
     <t>大細目，懸低耳。</t>
   </si>
   <si>
-    <t>P008</t>
+    <t>CAP008</t>
   </si>
   <si>
     <t>翁親某親，老婆仔拋捙輪。</t>
@@ -215,7 +215,7 @@
     <t>聽某喙，大富貴。</t>
   </si>
   <si>
-    <t>P009</t>
+    <t>CAP009</t>
   </si>
   <si>
     <t>菜蟲食菜，菜跤死。</t>
@@ -277,7 +277,7 @@
     <t>人牽毋行，鬼牽溜溜行。</t>
   </si>
   <si>
-    <t>P010</t>
+    <t>CAP010</t>
   </si>
   <si>
     <t>牛牢內觸牛母。</t>
@@ -320,7 +320,7 @@
     </r>
   </si>
   <si>
-    <t>P011</t>
+    <t>CAP011</t>
   </si>
   <si>
     <t>兄弟若仝心，烏塗變成金。</t>
@@ -336,7 +336,7 @@
     <t>飼囝無論飯，飼爸母算頓。</t>
   </si>
   <si>
-    <t>P012</t>
+    <t>CAP012</t>
   </si>
   <si>
     <t>船過水無痕。</t>
@@ -353,7 +353,7 @@
     <t>歹船拄著好港路。</t>
   </si>
   <si>
-    <t>P013</t>
+    <t>CAP013</t>
   </si>
   <si>
     <t>一樣米飼百樣人。</t>
@@ -367,7 +367,7 @@
     <t>五色人，講十色話。</t>
   </si>
   <si>
-    <t>P014</t>
+    <t>CAP014</t>
   </si>
   <si>
     <t>一喙掛雙舌。</t>
@@ -387,7 +387,7 @@
     <t>人濟話就濟，三色人講五色話。</t>
   </si>
   <si>
-    <t>P015</t>
+    <t>CAP015</t>
   </si>
   <si>
     <t>有樣看樣，無樣家己想。</t>
@@ -404,7 +404,7 @@
     <t>大狗盤牆，細狗看樣。</t>
   </si>
   <si>
-    <t>P016</t>
+    <t>CAP016</t>
   </si>
   <si>
     <t>一人一家代，公媽隨人祀。</t>
@@ -424,7 +424,7 @@
     <t>豬頭毋顧，顧鴨母卵。</t>
   </si>
   <si>
-    <t>P017</t>
+    <t>CAP017</t>
   </si>
   <si>
     <t>靠山山會崩，靠水水會焦。</t>
@@ -444,7 +444,7 @@
     <t>三分人，七分妝。</t>
   </si>
   <si>
-    <t>P018</t>
+    <t>CAP018</t>
   </si>
   <si>
     <t>橫柴夯入灶。</t>
@@ -467,7 +467,7 @@
     <t>臭頭仔嘛會做皇帝，做總統你嘛有機會。橫柴夯入灶。</t>
   </si>
   <si>
-    <t>P019</t>
+    <t>CAP019</t>
   </si>
   <si>
     <t>一斗較贏九石。</t>
@@ -487,7 +487,7 @@
     <t>俗物食破家。</t>
   </si>
   <si>
-    <t>P020</t>
+    <t>CAP020</t>
   </si>
   <si>
     <t>嫌貨才是買貨人。</t>
@@ -498,7 +498,7 @@
 </t>
   </si>
   <si>
-    <t>P021</t>
+    <t>CAP021</t>
   </si>
   <si>
     <t>有一好，無兩好。</t>
@@ -515,7 +515,7 @@
     <t>放屎也疼，放尿也疼。</t>
   </si>
   <si>
-    <t>P022</t>
+    <t>CAP022</t>
   </si>
   <si>
     <t>肉欲予人食，骨毋予人齧。</t>
@@ -532,7 +532,7 @@
     <t>舊囚食新囚。</t>
   </si>
   <si>
-    <t>P023</t>
+    <t>CAP023</t>
   </si>
   <si>
     <t>拍斷手骨顛倒勇。</t>
@@ -549,7 +549,7 @@
     <t>大格雞慢啼。</t>
   </si>
   <si>
-    <t>P024</t>
+    <t>CAP024</t>
   </si>
   <si>
     <t>戲棚跤徛久就是你的。</t>
@@ -566,7 +566,7 @@
     <t>三代粒積，一代窮空。</t>
   </si>
   <si>
-    <t>P025</t>
+    <t>CAP025</t>
   </si>
   <si>
     <t>老人囡仔性。</t>
@@ -586,7 +586,7 @@
     <t>囡仔人，大人心肝。</t>
   </si>
   <si>
-    <t>P026</t>
+    <t>CAP026</t>
   </si>
   <si>
     <t>做著歹田望下冬，娶著歹某一世人。</t>
@@ -603,7 +603,7 @@
     <t>買厝，買厝邊。</t>
   </si>
   <si>
-    <t>P027</t>
+    <t>CAP027</t>
   </si>
   <si>
     <t>戲館邊的豬母，袂歕簫嘛會拍拍。</t>
@@ -620,7 +620,7 @@
     <t>上山看山勢，入門看人意。</t>
   </si>
   <si>
-    <t>P028</t>
+    <t>CAP028</t>
   </si>
   <si>
     <t>欲好額等後世，欲做官學做戲。</t>
@@ -637,7 +637,7 @@
     <t>做官若清廉，食飯著攪鹽。</t>
   </si>
   <si>
-    <t>P029</t>
+    <t>CAP029</t>
   </si>
   <si>
     <t>龜跤趖出來。</t>
@@ -657,7 +657,7 @@
     <t>陰鴆陰鴆，咬人三寸深。</t>
   </si>
   <si>
-    <t>P030</t>
+    <t>CAP030</t>
   </si>
   <si>
     <t>幼秀跤，好命底。</t>
@@ -673,7 +673,7 @@
     <t>愛媠毋驚流鼻水。</t>
   </si>
   <si>
-    <t>P031</t>
+    <t>CAP031</t>
   </si>
   <si>
     <t>放屁安狗心。</t>
@@ -693,7 +693,7 @@
     <t>喙脣皮相款待。</t>
   </si>
   <si>
-    <t>P032</t>
+    <t>CAP032</t>
   </si>
   <si>
     <t>和尚頭掠蝨母。</t>
@@ -709,7 +709,7 @@
     <t>生狂狗食無屎。</t>
   </si>
   <si>
-    <t>P033</t>
+    <t>CAP033</t>
   </si>
   <si>
     <t>一鄉一俗。</t>
@@ -726,7 +726,7 @@
     <t>入人門，順人意。</t>
   </si>
   <si>
-    <t>P034</t>
+    <t>CAP034</t>
   </si>
   <si>
     <t>目睭掛斗概，看人物就愛。</t>
@@ -745,7 +745,7 @@
     <t>大碗閣滿墘。</t>
   </si>
   <si>
-    <t>P035</t>
+    <t>CAP035</t>
   </si>
   <si>
     <t>無日毋知晝，無鬚毋知老。</t>
@@ -765,7 +765,7 @@
     <t>等物僫到，等人快老。</t>
   </si>
   <si>
-    <t>P036</t>
+    <t>CAP036</t>
   </si>
   <si>
     <t>食人頭鍾酒，講人頭句話。</t>
@@ -778,7 +778,7 @@
     <t>關門著閂，講話著看。</t>
   </si>
   <si>
-    <t>P037</t>
+    <t>CAP037</t>
   </si>
   <si>
     <t>有狀元學生，無狀元先生。</t>
@@ -795,7 +795,7 @@
     <t>馬四跤也會著觸。</t>
   </si>
   <si>
-    <t>P038</t>
+    <t>CAP038</t>
   </si>
   <si>
     <t>相罵無揀喙，相拍無揀位。</t>
@@ -811,7 +811,7 @@
     <t>冤家變親家。</t>
   </si>
   <si>
-    <t>P039</t>
+    <t>CAP039</t>
   </si>
   <si>
     <t>雞屎落塗，也有三寸煙。</t>
@@ -822,7 +822,7 @@
 </t>
   </si>
   <si>
-    <t>P040</t>
+    <t>CAP040</t>
   </si>
   <si>
     <t>死蛇活尾溜。</t>
@@ -836,7 +836,7 @@
     <t>頭燒燒，尾冷冷。</t>
   </si>
   <si>
-    <t>P041</t>
+    <t>CAP041</t>
   </si>
   <si>
     <t>歹瓜厚子，歹人厚言語。</t>
@@ -847,7 +847,7 @@
 </t>
   </si>
   <si>
-    <t>P042</t>
+    <t>CAP042</t>
   </si>
   <si>
     <t>勸人做好代，較贏食早齋。</t>
@@ -867,7 +867,7 @@
     <t>好心好行，無衫通穿。</t>
   </si>
   <si>
-    <t>P043</t>
+    <t>CAP043</t>
   </si>
   <si>
     <t xml:space="preserve">Emma: "My parents have been putting most of their savings toward my education, even though it means giving up many things they want for themselves."
@@ -884,7 +884,7 @@
     <t>也著箠，也著糜。</t>
   </si>
   <si>
-    <t>P044</t>
+    <t>CAP044</t>
   </si>
   <si>
     <t>點油做記號。</t>
@@ -901,7 +901,7 @@
     <t>痟狗舂墓壙。</t>
   </si>
   <si>
-    <t>P045</t>
+    <t>CAP045</t>
   </si>
   <si>
     <t>入虎口，無死也烏漚。</t>
@@ -918,7 +918,7 @@
     <t>目睭看佇粿，跤踏著火。</t>
   </si>
   <si>
-    <t>P046</t>
+    <t>CAP046</t>
   </si>
   <si>
     <t>先顧腹肚，才顧佛祖。</t>
@@ -938,7 +938,7 @@
     <t>食飯皇帝大。</t>
   </si>
   <si>
-    <t>P047</t>
+    <t>CAP047</t>
   </si>
   <si>
     <t>外甥食母舅，親像食豆腐。</t>
@@ -955,7 +955,7 @@
     <t>手曲，屈入無屈出。</t>
   </si>
   <si>
-    <t>P048</t>
+    <t>CAP048</t>
   </si>
   <si>
     <t>胡蠅舞屎桮。</t>
@@ -974,7 +974,7 @@
     <t>乞食下大願。</t>
   </si>
   <si>
-    <t>P049</t>
+    <t>CAP049</t>
   </si>
   <si>
     <t xml:space="preserve">Maya: "My son wants to learn how to do all kinds of things, but I'm trying to choose activities that will actually be useful to him as he grows up."
@@ -985,7 +985,7 @@
     <t>王梨頭，西瓜尾。</t>
   </si>
   <si>
-    <t>P050</t>
+    <t>CAP050</t>
   </si>
   <si>
     <t>一句話三角六尖。</t>
@@ -996,7 +996,7 @@
 </t>
   </si>
   <si>
-    <t>P051</t>
+    <t>CAP051</t>
   </si>
   <si>
     <t>生的且一邊，養的恩情較大天。</t>
@@ -1016,7 +1016,7 @@
     <t>倖豬夯灶，倖囝不孝。</t>
   </si>
   <si>
-    <t>P052</t>
+    <t>CAP052</t>
   </si>
   <si>
     <t xml:space="preserve">Mia: "We were waiting for the guest speaker when we suddenly heard someone calling out loudly from the hallway."
@@ -1036,7 +1036,7 @@
     <t>五虎下西山。人未到，聲先到。</t>
   </si>
   <si>
-    <t>P053</t>
+    <t>CAP053</t>
   </si>
   <si>
     <t>一日走拋拋，一暝點燈膋。</t>
@@ -1066,7 +1066,7 @@
     </r>
   </si>
   <si>
-    <t>P054</t>
+    <t>CAP054</t>
   </si>
   <si>
     <t>忍氣求財，激氣相刣。</t>
@@ -1086,7 +1086,7 @@
     <t>好額毋值著會食，好命毋值著勇健。</t>
   </si>
   <si>
-    <t>P055</t>
+    <t>CAP055</t>
   </si>
   <si>
     <t xml:space="preserve">Maya: "I agreed to take charge of organizing the event, but now several things have gone wrong and everyone is looking to me to fix them."
@@ -1094,7 +1094,7 @@
 </t>
   </si>
   <si>
-    <t>P056</t>
+    <t>CAP056</t>
   </si>
   <si>
     <t xml:space="preserve">Emma: "He made a lot of money by taking advantage of people, but he spent most of it on gambling and lost nearly everything."
@@ -1102,7 +1102,7 @@
 </t>
   </si>
   <si>
-    <t>P057</t>
+    <t>CAP057</t>
   </si>
   <si>
     <t>上踏枋，上眠床，無洗跤睏中央。</t>
@@ -1119,7 +1119,7 @@
     <t>食米毋知米價</t>
   </si>
   <si>
-    <t>P058</t>
+    <t>CAP058</t>
   </si>
   <si>
     <t>囡仔人有耳無喙。</t>
@@ -1130,7 +1130,7 @@
 </t>
   </si>
   <si>
-    <t>P059</t>
+    <t>CAP059</t>
   </si>
   <si>
     <t>缺喙的食米粉──看現現。</t>
@@ -1150,7 +1150,7 @@
     <t>大紅花毋知䆀，圓仔花䆀毋知。</t>
   </si>
   <si>
-    <t>P060</t>
+    <t>CAP060</t>
   </si>
   <si>
     <t>神明興，弟子窮。</t>
@@ -1161,7 +1161,7 @@
 </t>
   </si>
   <si>
-    <t>P061</t>
+    <t>CAP061</t>
   </si>
   <si>
     <t>相分食有賰，相搶食無份。</t>
@@ -1172,7 +1172,7 @@
 </t>
   </si>
   <si>
-    <t>P062</t>
+    <t>CAP062</t>
   </si>
   <si>
     <t>狗無嫌主人散。</t>
@@ -1185,7 +1185,7 @@
     <t>明無轉厝，無祖；過年無轉厝，無某。</t>
   </si>
   <si>
-    <t>P063</t>
+    <t>CAP063</t>
   </si>
   <si>
     <t>功德做佇草仔埔。</t>
@@ -1199,7 +1199,7 @@
     <t>千算萬算，毋值天一劃。</t>
   </si>
   <si>
-    <t>P064</t>
+    <t>CAP064</t>
   </si>
   <si>
     <t xml:space="preserve">Mia: "I tried to fix the leaking sink myself, but somehow I ended up making the leak much worse and flooding part of the kitchen."
@@ -1213,7 +1213,7 @@
     <t>猴也會跋落樹跤。</t>
   </si>
   <si>
-    <t>P065</t>
+    <t>CAP065</t>
   </si>
   <si>
     <t xml:space="preserve">Mia: "I bought a pair of headphones online because they were much cheaper than the other brands, but they stopped working after a few days."
@@ -1221,7 +1221,7 @@
 </t>
   </si>
   <si>
-    <t>P066</t>
+    <t>CAP066</t>
   </si>
   <si>
     <t xml:space="preserve">Mia: "I bought a pineapple and a watermelon for the picnic, but I'm not sure which parts will taste the sweetest."
@@ -1235,7 +1235,7 @@
     <t>食米毋知米價。</t>
   </si>
   <si>
-    <t>P067</t>
+    <t>CAP067</t>
   </si>
   <si>
     <t xml:space="preserve">Maya: "Jason keeps jumping into every discussion, but he often struggles to explain what he means clearly."
@@ -1246,7 +1246,7 @@
     <t>乞食身，皇帝喙。</t>
   </si>
   <si>
-    <t>P068</t>
+    <t>CAP068</t>
   </si>
   <si>
     <t xml:space="preserve">Mia: "I've been practicing the piano for twenty minutes every day, even when I don't feel like it. After a few months, I can finally play pieces that used to seem impossible."
@@ -1260,7 +1260,7 @@
     <t>有燒香有保庇，有食藥有行氣。</t>
   </si>
   <si>
-    <t>P069</t>
+    <t>CAP069</t>
   </si>
   <si>
     <t xml:space="preserve">Mia: "We spent months preparing for the outdoor festival, but a sudden storm damaged the venue and forced us to cancel everything."
@@ -1268,14 +1268,14 @@
 </t>
   </si>
   <si>
-    <t>P070</t>
+    <t>CAP070</t>
   </si>
   <si>
     <t>Emma: "Whenever Jake sees his father sneaking extra food from the kitchen, he does the same thing when no one is watching."
 Ryan: "Kids really do pick up habits from the adults around them."</t>
   </si>
   <si>
-    <t>P071</t>
+    <t>CAP071</t>
   </si>
   <si>
     <r>
@@ -1318,7 +1318,7 @@
     <t>食著藥，青草一葉；食毋著藥，人參一石。</t>
   </si>
   <si>
-    <t>P072</t>
+    <t>CAP072</t>
   </si>
   <si>
     <t xml:space="preserve">Sophie: "The new intern just joined the company, but he's already telling the senior managers how they should run the entire department."
@@ -1326,7 +1326,7 @@
 </t>
   </si>
   <si>
-    <t>P073</t>
+    <t>CAP073</t>
   </si>
   <si>
     <t>清明無轉厝，無祖；過年無轉厝，無某。</t>
@@ -1340,7 +1340,7 @@
     <t>有唐山公，無唐山媽。</t>
   </si>
   <si>
-    <t>P074</t>
+    <t>CAP074</t>
   </si>
   <si>
     <t xml:space="preserve">Mia: "The department director barely acknowledges the junior staff and often dismisses their suggestions without listening to them."
@@ -1348,7 +1348,7 @@
 </t>
   </si>
   <si>
-    <t>P075</t>
+    <t>CAP075</t>
   </si>
   <si>
     <t xml:space="preserve">Emma: "I tried to finish the presentation as quickly as possible before the meeting, but I rushed through the final checks and accidentally sent the wrong version."
@@ -1356,7 +1356,7 @@
 </t>
   </si>
   <si>
-    <t>P076</t>
+    <t>CAP076</t>
   </si>
   <si>
     <t>臺灣錢，淹跤目。</t>
@@ -1373,7 +1373,7 @@
     <t>三百六十行，行行出狀元。</t>
   </si>
   <si>
-    <t>P077</t>
+    <t>CAP077</t>
   </si>
   <si>
     <t>夯石頭硩心肝。</t>
@@ -1384,7 +1384,7 @@
 </t>
   </si>
   <si>
-    <t>P078</t>
+    <t>CAP078</t>
   </si>
   <si>
     <t>人心肝，牛腹肚。</t>
@@ -1398,7 +1398,7 @@
     <t>睭掛斗概，看人物就愛。</t>
   </si>
   <si>
-    <t>P079</t>
+    <t>CAP079</t>
   </si>
   <si>
     <t xml:space="preserve">Emma: "We've tried several expensive marketing strategies, but none of them has helped increase sales. Maybe we're focusing on the wrong part of the problem."
@@ -1409,7 +1409,7 @@
     <t>江湖一點訣，講破毋值三仙錢。</t>
   </si>
   <si>
-    <t>P080</t>
+    <t>CAP080</t>
   </si>
   <si>
     <t>媠䆀無比止，愛著較慘死。</t>
@@ -1420,7 +1420,7 @@
 </t>
   </si>
   <si>
-    <t>P081</t>
+    <t>CAP081</t>
   </si>
   <si>
     <t xml:space="preserve">Emma: "My brother decided not to pursue a university degree and instead trained as a chef. He recently won a regional cooking competition."
@@ -1428,7 +1428,7 @@
 </t>
   </si>
   <si>
-    <t>P082</t>
+    <t>CAP082</t>
   </si>
   <si>
     <t xml:space="preserve">Anna: "My neighbor invited everyone over for a simple meal and spent the whole afternoon making sure everyone felt welcome."
@@ -1436,7 +1436,7 @@
 </t>
   </si>
   <si>
-    <t>P083</t>
+    <t>CAP083</t>
   </si>
   <si>
     <t>一某無人知，兩某相卸代。</t>
@@ -1449,7 +1449,7 @@
     <t>聽某喙，大富貴。一某無人知，兩某相卸代。</t>
   </si>
   <si>
-    <t>P084</t>
+    <t>CAP084</t>
   </si>
   <si>
     <t xml:space="preserve">Mia: "I'm getting to know my girlfriend's family, and I've noticed that her mother is very considerate and respectful toward everyone."
@@ -1457,7 +1457,7 @@
 </t>
   </si>
   <si>
-    <t>P085</t>
+    <t>CAP085</t>
   </si>
   <si>
     <t>一個囡仔較鬧熱三個大人。</t>
@@ -1473,7 +1473,7 @@
     <t>一肩擔雞，雙頭啼。</t>
   </si>
   <si>
-    <t>P086</t>
+    <t>CAP086</t>
   </si>
   <si>
     <t>食好鬥相報。</t>
@@ -1484,7 +1484,7 @@
 </t>
   </si>
   <si>
-    <t>P087</t>
+    <t>CAP087</t>
   </si>
   <si>
     <t xml:space="preserve">Mia: "My parents have always supported me, but I rarely visit them or help out when they need me."
@@ -1492,7 +1492,7 @@
 </t>
   </si>
   <si>
-    <t>P088</t>
+    <t>CAP088</t>
   </si>
   <si>
     <t xml:space="preserve">Sophie: "Mark just bought a new designer watch and keeps talking about how expensive it was, even though he complains about being short on money."
@@ -1500,7 +1500,7 @@
 </t>
   </si>
   <si>
-    <t>P089</t>
+    <t>CAP089</t>
   </si>
   <si>
     <t xml:space="preserve">Maya: "Everyone in the office keeps praising Lisa's new presentation, but she doesn't seem to realize how poorly she handled the questions afterward."
@@ -1508,7 +1508,7 @@
 </t>
   </si>
   <si>
-    <t>P090</t>
+    <t>CAP090</t>
   </si>
   <si>
     <t xml:space="preserve">Emma: "Our most experienced technician made a mistake while repairing the machine today, even though she's done this kind of work for years."
@@ -1516,14 +1516,14 @@
 </t>
   </si>
   <si>
-    <t>P091</t>
+    <t>CAP091</t>
   </si>
   <si>
     <t>Mia: "I thought repairing the old camera would require special expertise, but the technician showed me one simple adjustment that fixed the problem."
 Noah: "Sometimes something seems complicated until you know the key step."</t>
   </si>
   <si>
-    <t>P092</t>
+    <t>CAP092</t>
   </si>
   <si>
     <t xml:space="preserve">Olivia: "I've applied for several positions in my field, but none of the companies has offered me a job."
@@ -1531,7 +1531,7 @@
 </t>
   </si>
   <si>
-    <t>P093</t>
+    <t>CAP093</t>
   </si>
   <si>
     <t xml:space="preserve">Mia: "My wife suggested a different way to handle the budget, and it ended up saving us a lot of money."
@@ -1539,7 +1539,7 @@
 </t>
   </si>
   <si>
-    <t>P094</t>
+    <t>CAP094</t>
   </si>
   <si>
     <t xml:space="preserve">Maya: "My sister is raising two young children on her own while also working full-time to support the family. She spends most of her time trying to keep up with both responsibilities."
@@ -1550,7 +1550,7 @@
     <t>校長兼摃鐘。</t>
   </si>
   <si>
-    <t>P095</t>
+    <t>CAP095</t>
   </si>
   <si>
     <t xml:space="preserve">Emma: "I keep buying things online whenever I find a big discount, even when I don't really need them. My credit card bill has been getting harder to manage."
@@ -1558,7 +1558,7 @@
 </t>
   </si>
   <si>
-    <t>P096</t>
+    <t>CAP096</t>
   </si>
   <si>
     <t xml:space="preserve">Olivia: "I started learning how to bake, and my first few attempts were a complete mess. After practicing every weekend, I can finally make the recipes without much trouble."
@@ -1566,7 +1566,7 @@
 </t>
   </si>
   <si>
-    <t>P097</t>
+    <t>CAP097</t>
   </si>
   <si>
     <t xml:space="preserve">Maya: "My sister's baby is four months old, and the family is planning a small celebration for the occasion."
@@ -1577,21 +1577,21 @@
     <t>一个囡仔較鬧熱三个大人。</t>
   </si>
   <si>
-    <t>P098</t>
+    <t>CAP098</t>
   </si>
   <si>
     <t>Anna: "I thanked my host for dinner, but he insisted that I take some fruit home. When I declined, he brought out some homemade snacks instead."
 Michael: "He certainly doesn't want to let me leave without taking something."</t>
   </si>
   <si>
-    <t>P099</t>
+    <t>CAP099</t>
   </si>
   <si>
     <t>Mia: "I've been practicing for the certification exam every evening, even though progress has been slow. After several months, I finally passed."
 Daniel: "All that effort eventually paid off."</t>
   </si>
   <si>
-    <t>P100</t>
+    <t>CAP100</t>
   </si>
   <si>
     <t>揀啊揀，揀著一个賣龍眼。</t>
@@ -2887,7 +2887,7 @@
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="3" width="16.3516" style="1" customWidth="1"/>
-    <col min="4" max="4" width="46.9922" style="1" customWidth="1"/>
+    <col min="4" max="4" width="47" style="1" customWidth="1"/>
     <col min="5" max="9" width="16.3516" style="1" customWidth="1"/>
     <col min="10" max="16384" width="16.3516" style="1" customWidth="1"/>
   </cols>

</xml_diff>